<commit_message>
Removed loggers from each test method
</commit_message>
<xml_diff>
--- a/DataRetrieved/Languages.xlsx
+++ b/DataRetrieved/Languages.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="630" uniqueCount="137">
   <si>
     <t>Language</t>
   </si>
@@ -348,6 +348,81 @@
   </si>
   <si>
     <t>Tagalog</t>
+  </si>
+  <si>
+    <t>11,430</t>
+  </si>
+  <si>
+    <t>6,793</t>
+  </si>
+  <si>
+    <t>6,416</t>
+  </si>
+  <si>
+    <t>6,273</t>
+  </si>
+  <si>
+    <t>6,228</t>
+  </si>
+  <si>
+    <t>6,192</t>
+  </si>
+  <si>
+    <t>6,180</t>
+  </si>
+  <si>
+    <t>6,106</t>
+  </si>
+  <si>
+    <t>5,255</t>
+  </si>
+  <si>
+    <t>4,681</t>
+  </si>
+  <si>
+    <t>3,394</t>
+  </si>
+  <si>
+    <t>3,016</t>
+  </si>
+  <si>
+    <t>2,808</t>
+  </si>
+  <si>
+    <t>2,739</t>
+  </si>
+  <si>
+    <t>2,724</t>
+  </si>
+  <si>
+    <t>2,721</t>
+  </si>
+  <si>
+    <t>2,719</t>
+  </si>
+  <si>
+    <t>2,703</t>
+  </si>
+  <si>
+    <t>2,685</t>
+  </si>
+  <si>
+    <t>2,219</t>
+  </si>
+  <si>
+    <t>2,005</t>
+  </si>
+  <si>
+    <t>1,979</t>
+  </si>
+  <si>
+    <t>1,363</t>
+  </si>
+  <si>
+    <t>1,355</t>
+  </si>
+  <si>
+    <t>237</t>
   </si>
 </sst>
 </file>
@@ -408,7 +483,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>3</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3">
@@ -416,7 +491,7 @@
         <v>4</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>5</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4">
@@ -424,7 +499,7 @@
         <v>6</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>7</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5">
@@ -432,7 +507,7 @@
         <v>8</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>9</v>
+        <v>115</v>
       </c>
     </row>
     <row r="6">
@@ -440,7 +515,7 @@
         <v>10</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>11</v>
+        <v>116</v>
       </c>
     </row>
     <row r="7">
@@ -448,7 +523,7 @@
         <v>12</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>13</v>
+        <v>117</v>
       </c>
     </row>
     <row r="8">
@@ -456,7 +531,7 @@
         <v>14</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>15</v>
+        <v>118</v>
       </c>
     </row>
     <row r="9">
@@ -464,7 +539,7 @@
         <v>16</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>17</v>
+        <v>119</v>
       </c>
     </row>
     <row r="10">
@@ -472,7 +547,7 @@
         <v>18</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>19</v>
+        <v>120</v>
       </c>
     </row>
     <row r="11">
@@ -488,7 +563,7 @@
         <v>22</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>23</v>
+        <v>121</v>
       </c>
     </row>
     <row r="13">
@@ -496,7 +571,7 @@
         <v>24</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>25</v>
+        <v>122</v>
       </c>
     </row>
     <row r="14">
@@ -504,7 +579,7 @@
         <v>26</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>27</v>
+        <v>123</v>
       </c>
     </row>
     <row r="15">
@@ -528,7 +603,7 @@
         <v>32</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>33</v>
+        <v>124</v>
       </c>
     </row>
     <row r="18">
@@ -544,7 +619,7 @@
         <v>36</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>37</v>
+        <v>125</v>
       </c>
     </row>
     <row r="20">
@@ -552,7 +627,7 @@
         <v>38</v>
       </c>
       <c r="B20" t="s" s="0">
-        <v>39</v>
+        <v>126</v>
       </c>
     </row>
     <row r="21">
@@ -560,7 +635,7 @@
         <v>40</v>
       </c>
       <c r="B21" t="s" s="0">
-        <v>41</v>
+        <v>127</v>
       </c>
     </row>
     <row r="22">
@@ -568,7 +643,7 @@
         <v>42</v>
       </c>
       <c r="B22" t="s" s="0">
-        <v>43</v>
+        <v>128</v>
       </c>
     </row>
     <row r="23">
@@ -576,7 +651,7 @@
         <v>44</v>
       </c>
       <c r="B23" t="s" s="0">
-        <v>45</v>
+        <v>129</v>
       </c>
     </row>
     <row r="24">
@@ -584,7 +659,7 @@
         <v>46</v>
       </c>
       <c r="B24" t="s" s="0">
-        <v>47</v>
+        <v>130</v>
       </c>
     </row>
     <row r="25">
@@ -592,7 +667,7 @@
         <v>48</v>
       </c>
       <c r="B25" t="s" s="0">
-        <v>49</v>
+        <v>131</v>
       </c>
     </row>
     <row r="26">
@@ -600,7 +675,7 @@
         <v>50</v>
       </c>
       <c r="B26" t="s" s="0">
-        <v>51</v>
+        <v>132</v>
       </c>
     </row>
     <row r="27">
@@ -608,7 +683,7 @@
         <v>52</v>
       </c>
       <c r="B27" t="s" s="0">
-        <v>53</v>
+        <v>133</v>
       </c>
     </row>
     <row r="28">
@@ -616,7 +691,7 @@
         <v>54</v>
       </c>
       <c r="B28" t="s" s="0">
-        <v>55</v>
+        <v>134</v>
       </c>
     </row>
     <row r="29">
@@ -624,7 +699,7 @@
         <v>56</v>
       </c>
       <c r="B29" t="s" s="0">
-        <v>57</v>
+        <v>135</v>
       </c>
     </row>
     <row r="30">
@@ -632,7 +707,7 @@
         <v>58</v>
       </c>
       <c r="B30" t="s" s="0">
-        <v>59</v>
+        <v>136</v>
       </c>
     </row>
     <row r="31">
@@ -640,7 +715,7 @@
         <v>60</v>
       </c>
       <c r="B31" t="s" s="0">
-        <v>61</v>
+        <v>136</v>
       </c>
     </row>
     <row r="32">
@@ -717,23 +792,23 @@
     </row>
     <row r="41">
       <c r="A41" t="s" s="0">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B41" t="s" s="0">
-        <v>78</v>
+        <v>81</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="0">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B42" t="s" s="0">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s" s="0">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B43" t="s" s="0">
         <v>83</v>

</xml_diff>